<commit_message>
Reference the columns from another workbook using power query(Merge queries)
</commit_message>
<xml_diff>
--- a/Excel/Project/Freshmart/Cleaned/Cleaned_FreshMart_Employess.xlsx
+++ b/Excel/Project/Freshmart/Cleaned/Cleaned_FreshMart_Employess.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/AB6FF4EDD41B64DB/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{888251EE-B3E3-4A60-BA06-2E6DD13403ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D9E246E-25A2-49FA-B35A-7D261A2150F0}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{9A638044-DD53-4684-B3D4-457361A492B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77EB02C2-5C08-4DD9-8DD9-AA8410230FA9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B05D5C01-2CD9-4710-A107-1E4B8308DC9C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B05D5C01-2CD9-4710-A107-1E4B8308DC9C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Employees" sheetId="1" r:id="rId1"/>
+    <sheet name="Data_Profiling" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2133" uniqueCount="894">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2134" uniqueCount="895">
   <si>
     <t>Active</t>
   </si>
@@ -2713,13 +2713,16 @@
     <t>Using Ctrl+H</t>
   </si>
   <si>
-    <t>Change using Text to columns and change the format or use power query or use format cells</t>
-  </si>
-  <si>
     <t>Store_id</t>
   </si>
   <si>
     <t>Employee_status</t>
+  </si>
+  <si>
+    <t>Replaced Rs with Blanks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace using formats </t>
   </si>
 </sst>
 </file>
@@ -2809,47 +2812,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF1F4E78"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2988,6 +2950,47 @@
         <scheme val="none"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F4E78"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3002,17 +3005,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E5680E42-4237-49E6-93BD-87F83E54747B}" name="Table1" displayName="Table1" ref="A1:H351" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E5680E42-4237-49E6-93BD-87F83E54747B}" name="Employee" displayName="Employee" ref="A1:H351" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:H351" xr:uid="{E5680E42-4237-49E6-93BD-87F83E54747B}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9A91950F-30B2-4FB6-810A-2AD96D362C0B}" name="Employee_ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{980E9C3C-B431-4050-9A0B-1505AC9347D3}" name="Employee_Name" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{AFA55DEC-6DDF-4D22-9E06-1E158F077178}" name="Gender" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{97C2A0B3-3B5A-4BE9-9DE1-9FA612467720}" name="Department" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{8FEFD4EE-2E8C-44B0-9967-F7751C5947BF}" name="Salary" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{0D2936E5-423E-4C79-9606-4B0F1732FCD7}" name="Joining_Date" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{570BACBB-A687-49FC-8CBF-945D8C145447}" name="Store_ID" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{1330036D-CF6E-418E-AE92-D31E9366C952}" name="Employment_Status" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9A91950F-30B2-4FB6-810A-2AD96D362C0B}" name="Employee_ID" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{980E9C3C-B431-4050-9A0B-1505AC9347D3}" name="Employee_Name" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{AFA55DEC-6DDF-4D22-9E06-1E158F077178}" name="Gender" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{97C2A0B3-3B5A-4BE9-9DE1-9FA612467720}" name="Department" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{8FEFD4EE-2E8C-44B0-9967-F7751C5947BF}" name="Salary" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{0D2936E5-423E-4C79-9606-4B0F1732FCD7}" name="Joining_Date" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{570BACBB-A687-49FC-8CBF-945D8C145447}" name="Store_ID" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{1330036D-CF6E-418E-AE92-D31E9366C952}" name="Employment_Status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3336,19 +3339,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51809383-7272-432D-8411-0699A3FCA531}">
   <dimension ref="A1:H351"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="19.90625" customWidth="1"/>
-    <col min="5" max="5" width="20.54296875" customWidth="1"/>
-    <col min="6" max="6" width="17.36328125" customWidth="1"/>
-    <col min="7" max="7" width="16.90625" customWidth="1"/>
-    <col min="8" max="8" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>881</v>
       </c>
@@ -3374,7 +3377,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>873</v>
       </c>
@@ -3400,7 +3403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>871</v>
       </c>
@@ -3426,7 +3429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>869</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>867</v>
       </c>
@@ -3478,7 +3481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>865</v>
       </c>
@@ -3504,7 +3507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>863</v>
       </c>
@@ -3530,7 +3533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>861</v>
       </c>
@@ -3556,7 +3559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>859</v>
       </c>
@@ -3582,7 +3585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>857</v>
       </c>
@@ -3608,7 +3611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>854</v>
       </c>
@@ -3634,7 +3637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>852</v>
       </c>
@@ -3660,7 +3663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>850</v>
       </c>
@@ -3686,7 +3689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>848</v>
       </c>
@@ -3712,7 +3715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>846</v>
       </c>
@@ -3738,7 +3741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>844</v>
       </c>
@@ -3764,7 +3767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>842</v>
       </c>
@@ -3790,7 +3793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>840</v>
       </c>
@@ -3816,7 +3819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>838</v>
       </c>
@@ -3842,7 +3845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>836</v>
       </c>
@@ -3866,7 +3869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>834</v>
       </c>
@@ -3892,7 +3895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>831</v>
       </c>
@@ -3918,7 +3921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>829</v>
       </c>
@@ -3944,7 +3947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>827</v>
       </c>
@@ -3970,7 +3973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>825</v>
       </c>
@@ -3996,7 +3999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>823</v>
       </c>
@@ -4022,7 +4025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>821</v>
       </c>
@@ -4048,7 +4051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>819</v>
       </c>
@@ -4074,7 +4077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>817</v>
       </c>
@@ -4100,7 +4103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>815</v>
       </c>
@@ -4126,7 +4129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>813</v>
       </c>
@@ -4152,7 +4155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>810</v>
       </c>
@@ -4178,7 +4181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>808</v>
       </c>
@@ -4204,7 +4207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>806</v>
       </c>
@@ -4230,7 +4233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>804</v>
       </c>
@@ -4256,7 +4259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>802</v>
       </c>
@@ -4282,7 +4285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>800</v>
       </c>
@@ -4308,7 +4311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>798</v>
       </c>
@@ -4334,7 +4337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>796</v>
       </c>
@@ -4360,7 +4363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>793</v>
       </c>
@@ -4386,7 +4389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>791</v>
       </c>
@@ -4412,7 +4415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>789</v>
       </c>
@@ -4438,7 +4441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>787</v>
       </c>
@@ -4464,7 +4467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>785</v>
       </c>
@@ -4490,7 +4493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>782</v>
       </c>
@@ -4516,7 +4519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>778</v>
       </c>
@@ -4542,7 +4545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>776</v>
       </c>
@@ -4568,7 +4571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>774</v>
       </c>
@@ -4594,7 +4597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>771</v>
       </c>
@@ -4620,7 +4623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>768</v>
       </c>
@@ -4644,7 +4647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>767</v>
       </c>
@@ -4670,7 +4673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>765</v>
       </c>
@@ -4696,7 +4699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>763</v>
       </c>
@@ -4722,7 +4725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>761</v>
       </c>
@@ -4748,7 +4751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>759</v>
       </c>
@@ -4774,7 +4777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>757</v>
       </c>
@@ -4800,7 +4803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>755</v>
       </c>
@@ -4826,7 +4829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>753</v>
       </c>
@@ -4852,7 +4855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>751</v>
       </c>
@@ -4878,7 +4881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>748</v>
       </c>
@@ -4904,7 +4907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>746</v>
       </c>
@@ -4930,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>744</v>
       </c>
@@ -4956,7 +4959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>741</v>
       </c>
@@ -4982,7 +4985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>739</v>
       </c>
@@ -5008,7 +5011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>736</v>
       </c>
@@ -5034,7 +5037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>734</v>
       </c>
@@ -5060,7 +5063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>732</v>
       </c>
@@ -5086,7 +5089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>730</v>
       </c>
@@ -5112,7 +5115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>728</v>
       </c>
@@ -5138,7 +5141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>725</v>
       </c>
@@ -5164,7 +5167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>723</v>
       </c>
@@ -5190,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>720</v>
       </c>
@@ -5216,7 +5219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>718</v>
       </c>
@@ -5242,7 +5245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>716</v>
       </c>
@@ -5268,7 +5271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>713</v>
       </c>
@@ -5294,7 +5297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>710</v>
       </c>
@@ -5320,7 +5323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>707</v>
       </c>
@@ -5346,7 +5349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>705</v>
       </c>
@@ -5372,7 +5375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>703</v>
       </c>
@@ -5398,7 +5401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>700</v>
       </c>
@@ -5424,7 +5427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>698</v>
       </c>
@@ -5448,7 +5451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>696</v>
       </c>
@@ -5474,7 +5477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>694</v>
       </c>
@@ -5500,7 +5503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>692</v>
       </c>
@@ -5526,7 +5529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>690</v>
       </c>
@@ -5552,7 +5555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>688</v>
       </c>
@@ -5578,7 +5581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>686</v>
       </c>
@@ -5604,7 +5607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>684</v>
       </c>
@@ -5630,7 +5633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>682</v>
       </c>
@@ -5656,7 +5659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>680</v>
       </c>
@@ -5682,7 +5685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>677</v>
       </c>
@@ -5708,7 +5711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>675</v>
       </c>
@@ -5734,7 +5737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>673</v>
       </c>
@@ -5760,7 +5763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>670</v>
       </c>
@@ -5786,7 +5789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>668</v>
       </c>
@@ -5812,7 +5815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>666</v>
       </c>
@@ -5838,7 +5841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>664</v>
       </c>
@@ -5864,7 +5867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>662</v>
       </c>
@@ -5890,7 +5893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>660</v>
       </c>
@@ -5916,7 +5919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>658</v>
       </c>
@@ -5942,7 +5945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>656</v>
       </c>
@@ -5968,7 +5971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>654</v>
       </c>
@@ -5994,7 +5997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>652</v>
       </c>
@@ -6020,7 +6023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>650</v>
       </c>
@@ -6046,7 +6049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>648</v>
       </c>
@@ -6072,7 +6075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>645</v>
       </c>
@@ -6098,7 +6101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>642</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>640</v>
       </c>
@@ -6150,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>637</v>
       </c>
@@ -6176,7 +6179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>635</v>
       </c>
@@ -6202,7 +6205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>633</v>
       </c>
@@ -6228,7 +6231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>630</v>
       </c>
@@ -6254,7 +6257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>627</v>
       </c>
@@ -6280,7 +6283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>625</v>
       </c>
@@ -6306,7 +6309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>623</v>
       </c>
@@ -6332,7 +6335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>621</v>
       </c>
@@ -6358,7 +6361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>618</v>
       </c>
@@ -6384,7 +6387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>616</v>
       </c>
@@ -6410,7 +6413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>614</v>
       </c>
@@ -6436,7 +6439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>612</v>
       </c>
@@ -6462,7 +6465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>610</v>
       </c>
@@ -6488,7 +6491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>608</v>
       </c>
@@ -6514,7 +6517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>606</v>
       </c>
@@ -6540,7 +6543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>604</v>
       </c>
@@ -6566,7 +6569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>602</v>
       </c>
@@ -6592,7 +6595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>599</v>
       </c>
@@ -6618,7 +6621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>597</v>
       </c>
@@ -6644,7 +6647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>594</v>
       </c>
@@ -6670,7 +6673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>592</v>
       </c>
@@ -6696,7 +6699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>590</v>
       </c>
@@ -6722,7 +6725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>588</v>
       </c>
@@ -6748,7 +6751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>586</v>
       </c>
@@ -6774,7 +6777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>583</v>
       </c>
@@ -6800,7 +6803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>581</v>
       </c>
@@ -6826,7 +6829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>579</v>
       </c>
@@ -6852,7 +6855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>576</v>
       </c>
@@ -6878,7 +6881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>574</v>
       </c>
@@ -6904,7 +6907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>572</v>
       </c>
@@ -6930,7 +6933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>570</v>
       </c>
@@ -6956,7 +6959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>567</v>
       </c>
@@ -6982,7 +6985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>565</v>
       </c>
@@ -7008,7 +7011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>563</v>
       </c>
@@ -7034,7 +7037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>560</v>
       </c>
@@ -7060,7 +7063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>557</v>
       </c>
@@ -7086,7 +7089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>553</v>
       </c>
@@ -7112,7 +7115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>551</v>
       </c>
@@ -7138,7 +7141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>548</v>
       </c>
@@ -7164,7 +7167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>546</v>
       </c>
@@ -7190,7 +7193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>544</v>
       </c>
@@ -7216,7 +7219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>541</v>
       </c>
@@ -7242,7 +7245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>539</v>
       </c>
@@ -7268,7 +7271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>536</v>
       </c>
@@ -7294,7 +7297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>534</v>
       </c>
@@ -7320,7 +7323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>532</v>
       </c>
@@ -7346,7 +7349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>530</v>
       </c>
@@ -7372,7 +7375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>527</v>
       </c>
@@ -7398,7 +7401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>525</v>
       </c>
@@ -7424,7 +7427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>523</v>
       </c>
@@ -7450,7 +7453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>520</v>
       </c>
@@ -7476,7 +7479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>518</v>
       </c>
@@ -7502,7 +7505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>515</v>
       </c>
@@ -7528,7 +7531,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>512</v>
       </c>
@@ -7554,7 +7557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>510</v>
       </c>
@@ -7580,7 +7583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>508</v>
       </c>
@@ -7606,7 +7609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>506</v>
       </c>
@@ -7632,7 +7635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>504</v>
       </c>
@@ -7658,7 +7661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>502</v>
       </c>
@@ -7684,7 +7687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>500</v>
       </c>
@@ -7710,7 +7713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>498</v>
       </c>
@@ -7736,7 +7739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>496</v>
       </c>
@@ -7762,7 +7765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>494</v>
       </c>
@@ -7788,7 +7791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>491</v>
       </c>
@@ -7814,7 +7817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>489</v>
       </c>
@@ -7840,7 +7843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>487</v>
       </c>
@@ -7866,7 +7869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>484</v>
       </c>
@@ -7892,7 +7895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>481</v>
       </c>
@@ -7918,7 +7921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>478</v>
       </c>
@@ -7944,7 +7947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>476</v>
       </c>
@@ -7970,7 +7973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>473</v>
       </c>
@@ -7996,7 +7999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>471</v>
       </c>
@@ -8022,7 +8025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>469</v>
       </c>
@@ -8048,7 +8051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>466</v>
       </c>
@@ -8074,7 +8077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>464</v>
       </c>
@@ -8100,7 +8103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>462</v>
       </c>
@@ -8126,7 +8129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>459</v>
       </c>
@@ -8152,7 +8155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>457</v>
       </c>
@@ -8178,7 +8181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>454</v>
       </c>
@@ -8204,7 +8207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>452</v>
       </c>
@@ -8230,7 +8233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>449</v>
       </c>
@@ -8256,7 +8259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>447</v>
       </c>
@@ -8282,7 +8285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>445</v>
       </c>
@@ -8308,7 +8311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>442</v>
       </c>
@@ -8334,7 +8337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>439</v>
       </c>
@@ -8360,7 +8363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>436</v>
       </c>
@@ -8386,7 +8389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>434</v>
       </c>
@@ -8412,7 +8415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>431</v>
       </c>
@@ -8438,7 +8441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>429</v>
       </c>
@@ -8464,7 +8467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>426</v>
       </c>
@@ -8490,7 +8493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>424</v>
       </c>
@@ -8516,7 +8519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>421</v>
       </c>
@@ -8542,7 +8545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>418</v>
       </c>
@@ -8568,7 +8571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>414</v>
       </c>
@@ -8594,7 +8597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>411</v>
       </c>
@@ -8620,7 +8623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>408</v>
       </c>
@@ -8646,7 +8649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>406</v>
       </c>
@@ -8672,7 +8675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>403</v>
       </c>
@@ -8698,7 +8701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>401</v>
       </c>
@@ -8724,7 +8727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>399</v>
       </c>
@@ -8750,7 +8753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>396</v>
       </c>
@@ -8776,7 +8779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>394</v>
       </c>
@@ -8802,7 +8805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>391</v>
       </c>
@@ -8828,7 +8831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>389</v>
       </c>
@@ -8854,7 +8857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>387</v>
       </c>
@@ -8880,7 +8883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>384</v>
       </c>
@@ -8906,7 +8909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>382</v>
       </c>
@@ -8932,7 +8935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>379</v>
       </c>
@@ -8958,7 +8961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>376</v>
       </c>
@@ -8984,7 +8987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>374</v>
       </c>
@@ -9010,7 +9013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>371</v>
       </c>
@@ -9034,7 +9037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>370</v>
       </c>
@@ -9060,7 +9063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>367</v>
       </c>
@@ -9086,7 +9089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>365</v>
       </c>
@@ -9112,7 +9115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>362</v>
       </c>
@@ -9138,7 +9141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>358</v>
       </c>
@@ -9164,7 +9167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>355</v>
       </c>
@@ -9190,7 +9193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>352</v>
       </c>
@@ -9216,7 +9219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>349</v>
       </c>
@@ -9242,7 +9245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>347</v>
       </c>
@@ -9268,7 +9271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>344</v>
       </c>
@@ -9294,7 +9297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>342</v>
       </c>
@@ -9320,7 +9323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
         <v>339</v>
       </c>
@@ -9346,7 +9349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>337</v>
       </c>
@@ -9372,7 +9375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>334</v>
       </c>
@@ -9398,7 +9401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>331</v>
       </c>
@@ -9424,7 +9427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>329</v>
       </c>
@@ -9450,7 +9453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
         <v>327</v>
       </c>
@@ -9476,7 +9479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
         <v>325</v>
       </c>
@@ -9502,7 +9505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
         <v>322</v>
       </c>
@@ -9528,7 +9531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
         <v>320</v>
       </c>
@@ -9554,7 +9557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
         <v>317</v>
       </c>
@@ -9580,7 +9583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>314</v>
       </c>
@@ -9606,7 +9609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>312</v>
       </c>
@@ -9632,7 +9635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>310</v>
       </c>
@@ -9658,7 +9661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>308</v>
       </c>
@@ -9684,7 +9687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
         <v>305</v>
       </c>
@@ -9710,7 +9713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
         <v>302</v>
       </c>
@@ -9736,7 +9739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>300</v>
       </c>
@@ -9762,7 +9765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>298</v>
       </c>
@@ -9788,7 +9791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
         <v>295</v>
       </c>
@@ -9814,7 +9817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>293</v>
       </c>
@@ -9840,7 +9843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>291</v>
       </c>
@@ -9866,7 +9869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
         <v>288</v>
       </c>
@@ -9892,7 +9895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>285</v>
       </c>
@@ -9918,7 +9921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
         <v>282</v>
       </c>
@@ -9944,7 +9947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
         <v>279</v>
       </c>
@@ -9970,7 +9973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>277</v>
       </c>
@@ -9996,7 +9999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>274</v>
       </c>
@@ -10022,7 +10025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
         <v>272</v>
       </c>
@@ -10048,7 +10051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
         <v>270</v>
       </c>
@@ -10074,7 +10077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
         <v>268</v>
       </c>
@@ -10100,7 +10103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>265</v>
       </c>
@@ -10126,7 +10129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
         <v>262</v>
       </c>
@@ -10152,7 +10155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>259</v>
       </c>
@@ -10178,7 +10181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
         <v>256</v>
       </c>
@@ -10204,7 +10207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
         <v>253</v>
       </c>
@@ -10230,7 +10233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>251</v>
       </c>
@@ -10256,7 +10259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
         <v>248</v>
       </c>
@@ -10282,7 +10285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>245</v>
       </c>
@@ -10308,7 +10311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>242</v>
       </c>
@@ -10334,7 +10337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
         <v>239</v>
       </c>
@@ -10360,7 +10363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
         <v>236</v>
       </c>
@@ -10386,7 +10389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
         <v>233</v>
       </c>
@@ -10412,7 +10415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
         <v>231</v>
       </c>
@@ -10438,7 +10441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>228</v>
       </c>
@@ -10464,7 +10467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>225</v>
       </c>
@@ -10490,7 +10493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>222</v>
       </c>
@@ -10514,7 +10517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
         <v>220</v>
       </c>
@@ -10540,7 +10543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
         <v>218</v>
       </c>
@@ -10566,7 +10569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
         <v>215</v>
       </c>
@@ -10592,7 +10595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
         <v>213</v>
       </c>
@@ -10618,7 +10621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
         <v>211</v>
       </c>
@@ -10644,7 +10647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
         <v>208</v>
       </c>
@@ -10670,7 +10673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>206</v>
       </c>
@@ -10696,7 +10699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>204</v>
       </c>
@@ -10722,7 +10725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
         <v>202</v>
       </c>
@@ -10748,7 +10751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
         <v>199</v>
       </c>
@@ -10774,7 +10777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
         <v>196</v>
       </c>
@@ -10800,7 +10803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
         <v>193</v>
       </c>
@@ -10826,7 +10829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
         <v>190</v>
       </c>
@@ -10852,7 +10855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
         <v>187</v>
       </c>
@@ -10878,7 +10881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
         <v>184</v>
       </c>
@@ -10904,7 +10907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>181</v>
       </c>
@@ -10930,7 +10933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
         <v>178</v>
       </c>
@@ -10956,7 +10959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
         <v>175</v>
       </c>
@@ -10982,7 +10985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
         <v>173</v>
       </c>
@@ -11008,7 +11011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
         <v>170</v>
       </c>
@@ -11034,7 +11037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
         <v>167</v>
       </c>
@@ -11060,7 +11063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
         <v>164</v>
       </c>
@@ -11086,7 +11089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
         <v>161</v>
       </c>
@@ -11112,7 +11115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
         <v>158</v>
       </c>
@@ -11138,7 +11141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
         <v>155</v>
       </c>
@@ -11164,7 +11167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
         <v>152</v>
       </c>
@@ -11190,7 +11193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
         <v>149</v>
       </c>
@@ -11216,7 +11219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
         <v>147</v>
       </c>
@@ -11242,7 +11245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>144</v>
       </c>
@@ -11268,7 +11271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>141</v>
       </c>
@@ -11294,7 +11297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
         <v>138</v>
       </c>
@@ -11320,7 +11323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
         <v>135</v>
       </c>
@@ -11346,7 +11349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>132</v>
       </c>
@@ -11372,7 +11375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
         <v>129</v>
       </c>
@@ -11398,7 +11401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>127</v>
       </c>
@@ -11424,7 +11427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>124</v>
       </c>
@@ -11450,7 +11453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A313" s="1" t="s">
         <v>121</v>
       </c>
@@ -11476,7 +11479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A314" s="1" t="s">
         <v>118</v>
       </c>
@@ -11502,7 +11505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A315" s="1" t="s">
         <v>115</v>
       </c>
@@ -11528,7 +11531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A316" s="1" t="s">
         <v>112</v>
       </c>
@@ -11554,7 +11557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A317" s="1" t="s">
         <v>109</v>
       </c>
@@ -11580,7 +11583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A318" s="1" t="s">
         <v>106</v>
       </c>
@@ -11606,7 +11609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A319" s="1" t="s">
         <v>103</v>
       </c>
@@ -11632,7 +11635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A320" s="1" t="s">
         <v>100</v>
       </c>
@@ -11658,7 +11661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A321" s="1" t="s">
         <v>97</v>
       </c>
@@ -11684,7 +11687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A322" s="1" t="s">
         <v>95</v>
       </c>
@@ -11710,7 +11713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A323" s="1" t="s">
         <v>93</v>
       </c>
@@ -11736,7 +11739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A324" s="1" t="s">
         <v>90</v>
       </c>
@@ -11762,7 +11765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A325" s="1" t="s">
         <v>87</v>
       </c>
@@ -11788,7 +11791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A326" s="1" t="s">
         <v>84</v>
       </c>
@@ -11814,7 +11817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A327" s="1" t="s">
         <v>81</v>
       </c>
@@ -11840,7 +11843,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A328" s="1" t="s">
         <v>77</v>
       </c>
@@ -11866,7 +11869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A329" s="1" t="s">
         <v>74</v>
       </c>
@@ -11892,7 +11895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A330" s="1" t="s">
         <v>71</v>
       </c>
@@ -11918,7 +11921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A331" s="1" t="s">
         <v>68</v>
       </c>
@@ -11944,7 +11947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A332" s="1" t="s">
         <v>65</v>
       </c>
@@ -11970,7 +11973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A333" s="1" t="s">
         <v>62</v>
       </c>
@@ -11996,7 +11999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A334" s="1" t="s">
         <v>59</v>
       </c>
@@ -12022,7 +12025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A335" s="1" t="s">
         <v>56</v>
       </c>
@@ -12048,7 +12051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A336" s="1" t="s">
         <v>53</v>
       </c>
@@ -12074,7 +12077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A337" s="1" t="s">
         <v>51</v>
       </c>
@@ -12100,7 +12103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A338" s="1" t="s">
         <v>48</v>
       </c>
@@ -12126,7 +12129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A339" s="1" t="s">
         <v>44</v>
       </c>
@@ -12152,7 +12155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A340" s="1" t="s">
         <v>41</v>
       </c>
@@ -12178,7 +12181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A341" s="1" t="s">
         <v>38</v>
       </c>
@@ -12204,7 +12207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A342" s="1" t="s">
         <v>35</v>
       </c>
@@ -12230,7 +12233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A343" s="1" t="s">
         <v>31</v>
       </c>
@@ -12256,7 +12259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A344" s="1" t="s">
         <v>28</v>
       </c>
@@ -12280,7 +12283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A345" s="1" t="s">
         <v>26</v>
       </c>
@@ -12306,7 +12309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A346" s="1" t="s">
         <v>23</v>
       </c>
@@ -12332,7 +12335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="347" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A347" s="1" t="s">
         <v>20</v>
       </c>
@@ -12358,7 +12361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A348" s="1" t="s">
         <v>17</v>
       </c>
@@ -12384,7 +12387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="349" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A349" s="1" t="s">
         <v>13</v>
       </c>
@@ -12410,7 +12413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A350" s="1" t="s">
         <v>9</v>
       </c>
@@ -12436,7 +12439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A351" s="1" t="s">
         <v>5</v>
       </c>
@@ -12473,15 +12476,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AADF1BD8-6510-4C42-B263-8034D1ECAE0D}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.81640625" customWidth="1"/>
-    <col min="2" max="2" width="14.81640625" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" customWidth="1"/>
-    <col min="4" max="4" width="65.36328125" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>882</v>
       </c>
@@ -12495,7 +12498,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>886</v>
       </c>
@@ -12509,7 +12512,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>879</v>
       </c>
@@ -12520,15 +12523,18 @@
         <v>890</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>877</v>
       </c>
       <c r="B4" t="s">
         <v>889</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D4" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>876</v>
       </c>
@@ -12536,12 +12542,12 @@
         <v>889</v>
       </c>
       <c r="D5" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>891</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>892</v>
       </c>
       <c r="B6" t="s">
         <v>887</v>
@@ -12553,9 +12559,9 @@
         <v>888</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B7" t="s">
         <v>889</v>

</xml_diff>